<commit_message>
GL-4 DPE_LISA_P1+DPE_LISA_P2 updated EDU_LEVEL
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/DPE_LISA_P1.xlsx
+++ b/rmonize/data_proc_elem/DPE_LISA_P1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F54842-1D9A-4767-9CAD-1E9759DCC8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C4AFFB-BF15-49AD-B498-31C3584DB89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22260" windowHeight="12000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11025" yWindow="0" windowWidth="11025" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_processing_elements_templa" sheetId="1" r:id="rId1"/>
@@ -1290,21 +1290,19 @@
   </si>
   <si>
     <t>case_when(
-      MUTBILD_0 == 1 &amp; VATBILD_0 == 1 ~ 0L,
-      MUTBILD_0 %in% c(2) | VATBILD_0 %in% c(2) ~ 1L,  
-      MUTBILD_0 %in% c(3) | VATBILD_0 %in% c(3) ~ 3L, 
-      MUTBILD_0 %in% c(4) | VATBILD_0 %in% c(4) ~ 2L, 
-      MUTBILD_0 %in% c(5, 6) | VATBILD_0 %in% c(5, 6) ~ 4L, 
-      MUTBILD_0 %in% c(7) | VATBILD_0 %in% c(7) ~ 5L,  
+      MUTBILD_0 %in% c(5, 6) | VATBILD_0 %in% c(5, 6) ~ 4L,
+      MUTBILD_0 %in% c(3,4) | VATBILD_0 %in% c(3,4) ~ 3L,
+      MUTBILD_0 %in% c(2) | VATBILD_0 %in% c(2) ~ 1L,
+      MUTBILD_0 == 1 | VATBILD_0 == 1 ~ 0L,
+      MUTBILD_0 %in% c(7) | VATBILD_0 %in% c(7) ~ 5L,
       TRUE ~ NA_integer_
     )</t>
   </si>
   <si>
-    <t>"None" (0): Both parents have 1 (no certificate).
+    <t>"Longer Education" (4): Either parent has 5 or 6.
+"Secondary School" (3): Either parent has 3 or 4.
 "Primary School Completed" (1): Either parent has 2.
-"Technical/Professional School" (2): Either parent has 4.
-"Secondary School" (3): Either parent has 3.
-"Longer Education" (4): Either parent has 5 or 6.
+"None" (0): Either parent has 1 (no certificate).
 "Not Specified" (5): Either parent has 7 (other degree).</t>
   </si>
 </sst>
@@ -1899,7 +1897,7 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2408,7 +2406,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="255" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -6459,6 +6457,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B1DC67C611DD5E4D81775F9F3E26A7B2" ma:contentTypeVersion="16" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7f379a5812b480a74f9d031be5f88a83">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xmlns:ns3="12535b08-222e-45d2-b6db-15019f1afee6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dbce1e37d7de67e1c835013ca0ee7a7c" ns2:_="" ns3:_="">
     <xsd:import namespace="b63cdcf7-47fa-43f6-87e5-23b415b5c413"/>
@@ -6699,15 +6706,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6721,6 +6719,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E89B3EC5-962B-41D9-9821-3A191D2434CD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA68FB6B-B5E6-4AB5-ACC7-06ACAB30D951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6735,14 +6741,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E89B3EC5-962B-41D9-9821-3A191D2434CD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>